<commit_message>
Publish Prague_2013_WCH, Pau_2017_WWC, Deodoro_2016_OG, LaPlagne_2012_WWC, DeepCreek_2014_WCH, Kasai_2021_OG
</commit_message>
<xml_diff>
--- a/events/Deodoro_2016_OG/Deodoro_2016_OG_start.xlsx
+++ b/events/Deodoro_2016_OG/Deodoro_2016_OG_start.xlsx
@@ -5424,7 +5424,12 @@
       </c>
       <c r="R86" t="inlineStr">
         <is>
-          <t>Borba M/Moraes C</t>
+          <t>Borba M</t>
+        </is>
+      </c>
+      <c r="S86" t="inlineStr">
+        <is>
+          <t>Moraes C</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5474,12 @@
       </c>
       <c r="R87" t="inlineStr">
         <is>
-          <t>Munhoz W/Vierra C</t>
+          <t>Munhoz W</t>
+        </is>
+      </c>
+      <c r="S87" t="inlineStr">
+        <is>
+          <t>Vierra C</t>
         </is>
       </c>
     </row>
@@ -12894,7 +12904,12 @@
       </c>
       <c r="R209" t="inlineStr">
         <is>
-          <t>Borba M/Moraes C</t>
+          <t>Borba M</t>
+        </is>
+      </c>
+      <c r="S209" t="inlineStr">
+        <is>
+          <t>Moraes C</t>
         </is>
       </c>
     </row>
@@ -12939,7 +12954,12 @@
       </c>
       <c r="R210" t="inlineStr">
         <is>
-          <t>Munhoz W/Vierra C</t>
+          <t>Munhoz W</t>
+        </is>
+      </c>
+      <c r="S210" t="inlineStr">
+        <is>
+          <t>Vierra C</t>
         </is>
       </c>
     </row>

</xml_diff>